<commit_message>
remove fineweb edu data from config 2023 wiki
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -1701,10 +1701,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:17">
       <c r="A1">
         <v>500</v>
       </c>
@@ -1735,8 +1735,23 @@
       <c r="K1">
         <v>-3.6864</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="M1">
+        <v>250</v>
+      </c>
+      <c r="N1" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="O1" s="1">
+        <v>0.912</v>
+      </c>
+      <c r="P1">
+        <v>-4.3833</v>
+      </c>
+      <c r="Q1">
+        <v>-3.3462</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>1000</v>
       </c>
@@ -1767,8 +1782,23 @@
       <c r="K2">
         <v>-3.4793</v>
       </c>
-    </row>
-    <row r="3" spans="1:11">
+      <c r="M2">
+        <v>500</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0.908</v>
+      </c>
+      <c r="P2">
+        <v>-4.1102</v>
+      </c>
+      <c r="Q2">
+        <v>-3.3407</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>1500</v>
       </c>
@@ -1799,8 +1829,23 @@
       <c r="K3">
         <v>-3.4828</v>
       </c>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="M3">
+        <v>750</v>
+      </c>
+      <c r="N3" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0.892</v>
+      </c>
+      <c r="P3">
+        <v>-4.1766</v>
+      </c>
+      <c r="Q3">
+        <v>-3.3397</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>2000</v>
       </c>
@@ -1831,8 +1876,23 @@
       <c r="K4">
         <v>-3.4507</v>
       </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="M4">
+        <v>1000</v>
+      </c>
+      <c r="N4" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0.912</v>
+      </c>
+      <c r="P4">
+        <v>-4.1182</v>
+      </c>
+      <c r="Q4">
+        <v>-3.3339</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>3000</v>
       </c>
@@ -1863,8 +1923,23 @@
       <c r="K5">
         <v>-3.6002</v>
       </c>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="M5">
+        <v>1250</v>
+      </c>
+      <c r="N5" s="1">
+        <v>0.85</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0.908</v>
+      </c>
+      <c r="P5">
+        <v>-4.5955</v>
+      </c>
+      <c r="Q5">
+        <v>-3.5169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>4000</v>
       </c>
@@ -1895,8 +1970,23 @@
       <c r="K6">
         <v>-3.6174</v>
       </c>
-    </row>
-    <row r="7" spans="1:11">
+      <c r="M6">
+        <v>1500</v>
+      </c>
+      <c r="N6" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="O6" s="1">
+        <v>0.888</v>
+      </c>
+      <c r="P6">
+        <v>-4.2559</v>
+      </c>
+      <c r="Q6">
+        <v>-3.6748</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>6000</v>
       </c>
@@ -1927,8 +2017,23 @@
       <c r="K7">
         <v>-3.8947</v>
       </c>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="M7">
+        <v>1750</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="O7" s="1">
+        <v>0.888</v>
+      </c>
+      <c r="P7">
+        <v>-4.6736</v>
+      </c>
+      <c r="Q7">
+        <v>-3.8438</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8">
         <v>7000</v>
       </c>
@@ -1959,8 +2064,23 @@
       <c r="K8">
         <v>-3.9759</v>
       </c>
-    </row>
-    <row r="9" spans="1:11">
+      <c r="M8">
+        <v>2000</v>
+      </c>
+      <c r="N8" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="O8" s="1">
+        <v>0.867</v>
+      </c>
+      <c r="P8">
+        <v>-4.7518</v>
+      </c>
+      <c r="Q8">
+        <v>-3.7646</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9">
         <v>8000</v>
       </c>
@@ -1991,8 +2111,23 @@
       <c r="K9">
         <v>-3.5343</v>
       </c>
-    </row>
-    <row r="10" spans="1:11">
+      <c r="M9">
+        <v>2250</v>
+      </c>
+      <c r="N9" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0.908</v>
+      </c>
+      <c r="P9">
+        <v>-4.246</v>
+      </c>
+      <c r="Q9">
+        <v>-3.5466</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10">
         <v>9000</v>
       </c>
@@ -2023,8 +2158,23 @@
       <c r="K10">
         <v>-3.2213</v>
       </c>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="M10">
+        <v>2500</v>
+      </c>
+      <c r="N10" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0.908</v>
+      </c>
+      <c r="P10">
+        <v>-4.2679</v>
+      </c>
+      <c r="Q10">
+        <v>-3.5801</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>10000</v>
       </c>
@@ -2056,7 +2206,7 @@
         <v>-3.2124</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>11000</v>
       </c>
@@ -2088,7 +2238,7 @@
         <v>-3.2884</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:17">
       <c r="A13">
         <v>12000</v>
       </c>
@@ -2120,7 +2270,7 @@
         <v>-3.4543</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:17">
       <c r="A14">
         <v>13000</v>
       </c>
@@ -2152,7 +2302,7 @@
         <v>-3.5854</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:17">
       <c r="A15">
         <v>13500</v>
       </c>
@@ -2184,7 +2334,7 @@
         <v>-3.5821</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:17">
       <c r="A16">
         <v>14000</v>
       </c>

</xml_diff>

<commit_message>
set weight 0.2, 0.8
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11100" activeTab="2"/>
+    <workbookView windowWidth="14010" windowHeight="5580" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="2021" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="10">
   <si>
     <t>post cutoff percent</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>Failed</t>
+  </si>
+  <si>
+    <t>2024 year</t>
   </si>
 </sst>
 </file>
@@ -1704,7 +1707,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V55"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:22">
@@ -3092,6 +3095,108 @@
       </c>
       <c r="E48">
         <v>-3.3756</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6">
+      <c r="A50" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6">
+      <c r="A51">
+        <v>1500</v>
+      </c>
+      <c r="B51" s="1">
+        <v>0.375</v>
+      </c>
+      <c r="C51" s="1">
+        <v>0.588</v>
+      </c>
+      <c r="D51">
+        <v>-12.2562</v>
+      </c>
+      <c r="E51">
+        <v>-11.2603</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6">
+      <c r="A52">
+        <v>3000</v>
+      </c>
+      <c r="B52" s="1">
+        <v>0.625</v>
+      </c>
+      <c r="C52" s="1">
+        <v>0.642</v>
+      </c>
+      <c r="D52">
+        <v>-9.6948</v>
+      </c>
+      <c r="E52">
+        <v>-10.2921</v>
+      </c>
+      <c r="F52" s="1">
+        <v>0.914</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6">
+      <c r="A53">
+        <v>4500</v>
+      </c>
+      <c r="B53" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="C53" s="1">
+        <v>0.733</v>
+      </c>
+      <c r="D53">
+        <v>-9.7527</v>
+      </c>
+      <c r="E53">
+        <v>-8.3458</v>
+      </c>
+      <c r="F53" s="1">
+        <v>0.8109</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6">
+      <c r="A54">
+        <v>6000</v>
+      </c>
+      <c r="B54" s="1">
+        <v>0.75</v>
+      </c>
+      <c r="C54" s="1">
+        <v>0.721</v>
+      </c>
+      <c r="D54">
+        <v>-8.8214</v>
+      </c>
+      <c r="E54">
+        <v>-7.1411</v>
+      </c>
+      <c r="F54" s="1">
+        <v>0.8556</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6">
+      <c r="A55">
+        <v>7500</v>
+      </c>
+      <c r="B55" s="1">
+        <v>0.825</v>
+      </c>
+      <c r="C55" s="1">
+        <v>0.783</v>
+      </c>
+      <c r="D55">
+        <v>-7.7781</v>
+      </c>
+      <c r="E55">
+        <v>-6.6901</v>
+      </c>
+      <c r="F55" s="1">
+        <v>0.9368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
modify config to use only cpt and fineweb
</commit_message>
<xml_diff>
--- a/test.xlsx
+++ b/test.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11100" activeTab="2"/>
+    <workbookView windowWidth="28800" windowHeight="11700" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="2021" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="12">
   <si>
     <t>post cutoff percent</t>
   </si>
@@ -64,6 +64,9 @@
   </si>
   <si>
     <t>cpt:0.8, fineweb:0.2</t>
+  </si>
+  <si>
+    <t>cpt: 0.95, category : 0.05</t>
   </si>
 </sst>
 </file>
@@ -3100,15 +3103,18 @@
         <v>-3.3756</v>
       </c>
     </row>
-    <row r="50" spans="1:12">
+    <row r="50" spans="1:18">
       <c r="A50" t="s">
         <v>9</v>
       </c>
       <c r="I50" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="51" spans="1:12">
+      <c r="N50" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18">
       <c r="A51">
         <v>1500</v>
       </c>
@@ -3139,8 +3145,23 @@
       <c r="L51">
         <v>-10.6389</v>
       </c>
-    </row>
-    <row r="52" spans="1:12">
+      <c r="N51">
+        <v>1000</v>
+      </c>
+      <c r="O51" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="P51" s="1">
+        <v>0.642</v>
+      </c>
+      <c r="Q51">
+        <v>-11.2652</v>
+      </c>
+      <c r="R51">
+        <v>-9.9791</v>
+      </c>
+    </row>
+    <row r="52" spans="1:18">
       <c r="A52">
         <v>3000</v>
       </c>
@@ -3159,6 +3180,9 @@
       <c r="F52" s="1">
         <v>0.914</v>
       </c>
+      <c r="H52">
+        <v>2000</v>
+      </c>
       <c r="I52" s="1">
         <v>0.625</v>
       </c>
@@ -3171,8 +3195,23 @@
       <c r="L52">
         <v>-9.2401</v>
       </c>
-    </row>
-    <row r="53" spans="1:12">
+      <c r="N52">
+        <v>2000</v>
+      </c>
+      <c r="O52" s="1">
+        <v>0.6</v>
+      </c>
+      <c r="P52" s="1">
+        <v>0.675</v>
+      </c>
+      <c r="Q52">
+        <v>-10.2443</v>
+      </c>
+      <c r="R52">
+        <v>-9.8982</v>
+      </c>
+    </row>
+    <row r="53" spans="1:18">
       <c r="A53">
         <v>4500</v>
       </c>
@@ -3191,8 +3230,23 @@
       <c r="F53" s="1">
         <v>0.8109</v>
       </c>
-    </row>
-    <row r="54" spans="1:12">
+      <c r="N53">
+        <v>3000</v>
+      </c>
+      <c r="O53" s="1">
+        <v>0.625</v>
+      </c>
+      <c r="P53" s="1">
+        <v>0.721</v>
+      </c>
+      <c r="Q53">
+        <v>-10.1317</v>
+      </c>
+      <c r="R53">
+        <v>-9.0458</v>
+      </c>
+    </row>
+    <row r="54" spans="1:18">
       <c r="A54">
         <v>6000</v>
       </c>
@@ -3211,8 +3265,23 @@
       <c r="F54" s="1">
         <v>0.8556</v>
       </c>
-    </row>
-    <row r="55" spans="1:12">
+      <c r="N54">
+        <v>4000</v>
+      </c>
+      <c r="O54" s="1">
+        <v>0.65</v>
+      </c>
+      <c r="P54" s="1">
+        <v>0.767</v>
+      </c>
+      <c r="Q54">
+        <v>-9.8482</v>
+      </c>
+      <c r="R54">
+        <v>-8.7919</v>
+      </c>
+    </row>
+    <row r="55" spans="1:18">
       <c r="A55">
         <v>7500</v>
       </c>

</xml_diff>